<commit_message>
Document Iwate machine-cost (損料) basis in dump truck cost workbook
Iwate applies the MLIT 建設機械等損料表 and classifies all cities as
heavy-snow B areas, so the snow-adjusted Niigata values remain the
closest public equivalent; add Iwate sources and replacement notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UpX1QaVcgm2gRXfCZCnaQB
</commit_message>
<xml_diff>
--- a/research/iwate_10t_dump_cost.xlsx
+++ b/research/iwate_10t_dump_cost.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="230" uniqueCount="179">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="185">
   <si>
     <r>
       <rPr>
@@ -1094,7 +1094,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">積級：年間運転</t>
+      <t xml:space="preserve">積級（豪雪補正後）：年間運転</t>
     </r>
     <r>
       <rPr>
@@ -1132,7 +1132,45 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">日</t>
+      <t xml:space="preserve">日。岩手</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">地区</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">も同条件</t>
     </r>
   </si>
   <si>
@@ -1294,26 +1332,45 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">同上 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">MNS0301005</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">（豪雪補正込、タイヤ損耗費及び補修費</t>
+      <t xml:space="preserve">新潟県農地部 機械損料一覧表</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(R7.10.20</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">適用</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) MNS0301005</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（豪雪補正込・タイヤ損耗費及び補修費</t>
     </r>
     <r>
       <rPr>
@@ -1351,7 +1408,83 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">含む）。岩手県版の損料表があれば置換</t>
+      <t xml:space="preserve">含む）。岩手県は独自の損料表を公表せず国交省『建設機械等損料表』を適用し、県内全市が豪雪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">地区（県積算基準 運用編 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">R8.10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）→豪雪補正込の本値と同じ扱い。令和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年度版の値は市販本（日本建設機械施工協会、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円）で確認し置換</t>
     </r>
   </si>
   <si>
@@ -2583,7 +2716,72 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">・損料は新潟県（豪雪補正込）の値で代用している。岩手県県土整備部・東北地方整備局の損料表があれば置き換えること。</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">・岩手県は損料表を独自公表しておらず、国交省『建設機械等損料表』を準用（県内全市は豪雪</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">地区）。本表は同じ国交省表に豪雪補正をかけて公表している新潟県（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">R7.10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">適用）の値を使用。令和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年度版の数値は市販本で確認して前提条件シートを置換すること。</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">・労務単価は賃金のみで、法定福利費の事業主負担は含まない（ここでは諸経費率に含めて計上）。</t>
@@ -3386,6 +3584,162 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.pref.niigata.lg.jp/uploaded/attachment/474671.pdf</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">岩手県 令和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年度土木工事標準積算基準書（公表用）※損料表は国交省版を適用</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pref.iwate.jp/kendozukuri/kensetsu/1093671/1101385.html</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">岩手県 土木工事標準積算基準書（運用編）令和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">月</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日以降適用 ※機械所在地の豪雪地域区分（岩手県全市＝</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">B</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">地区）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pref.iwate.jp/_res/projects/default_project/_page_/001/101/385/261001_unnyouhen.pdf</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日本建設機械施工協会『建設機械等損料表 令和</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年度版』（市販）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.gov-book.or.jp/book/detail.php?product_id=408304</t>
   </si>
   <si>
     <r>
@@ -5600,7 +5954,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -5657,7 +6011,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
         <v>172</v>
       </c>
@@ -5665,7 +6019,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
         <v>174</v>
       </c>
@@ -5673,20 +6027,44 @@
         <v>175</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>151</v>
+        <v>176</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>178</v>
+        <v>179</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="28" t="s">
+        <v>180</v>
+      </c>
+      <c r="B12" s="37" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="28" t="s">
+        <v>151</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="28" t="s">
+        <v>183</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>184</v>
       </c>
     </row>
   </sheetData>
@@ -5695,11 +6073,14 @@
     <hyperlink ref="B4" r:id="rId2" display="https://jta.or.jp/wp-content/themes/jta_theme/pdf/202410unchin.pdf"/>
     <hyperlink ref="B5" r:id="rId3" display="https://www.rinya.maff.go.jp/j/sekou/gijutu/attach/pdf/sekisan_kijun-374.pdf"/>
     <hyperlink ref="B6" r:id="rId4" display="https://www.pref.niigata.lg.jp/uploaded/attachment/474671.pdf"/>
-    <hyperlink ref="B7" r:id="rId5" display="https://www.rinya.maff.go.jp/tohoku/apply/publicsale/iwatenanbu/attach/pdf/tya-ta-2-5.pdf"/>
-    <hyperlink ref="B8" r:id="rId6" display="https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html"/>
-    <hyperlink ref="B9" r:id="rId7" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
-    <hyperlink ref="B10" r:id="rId8" display="https://www.matsudakougyou.com/price/"/>
-    <hyperlink ref="B11" r:id="rId9" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
+    <hyperlink ref="B7" r:id="rId5" display="https://www.pref.iwate.jp/kendozukuri/kensetsu/1093671/1101385.html"/>
+    <hyperlink ref="B8" r:id="rId6" display="https://www.pref.iwate.jp/_res/projects/default_project/_page_/001/101/385/261001_unnyouhen.pdf"/>
+    <hyperlink ref="B9" r:id="rId7" display="https://www.gov-book.or.jp/book/detail.php?product_id=408304"/>
+    <hyperlink ref="B10" r:id="rId8" display="https://www.rinya.maff.go.jp/tohoku/apply/publicsale/iwatenanbu/attach/pdf/tya-ta-2-5.pdf"/>
+    <hyperlink ref="B11" r:id="rId9" display="https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html"/>
+    <hyperlink ref="B12" r:id="rId10" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
+    <hyperlink ref="B13" r:id="rId11" display="https://www.matsudakougyou.com/price/"/>
+    <hyperlink ref="B14" r:id="rId12" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Set new 10t dump truck price to 20M yen in cost workbook
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UpX1QaVcgm2gRXfCZCnaQB
</commit_message>
<xml_diff>
--- a/research/iwate_10t_dump_cost.xlsx
+++ b/research/iwate_10t_dump_cost.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
   <si>
     <r>
       <rPr>
@@ -377,17 +377,188 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">新潟県農地部 機械損料一覧表</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(R7.10.20</t>
+      <t xml:space="preserve">新車</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10t</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダンプの販売相場 税込約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1,800</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万〜</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2,500</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円（中心</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円前後：トラック流通センター、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GROOWAVE</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SIGMA</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">、販売店の</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2026</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">年式実例</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2,491</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円）を踏まえ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円と設定。参考：新潟県 機械損料一覧表</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(R7.10</t>
     </r>
     <r>
       <rPr>
@@ -406,16 +577,16 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">) 10t</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">積級ダンプ基礎価格 </t>
+      <t xml:space="preserve">)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">の積算用基礎価格は</t>
     </r>
     <r>
       <rPr>
@@ -434,7 +605,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">千円 に付属品等を加味</t>
+      <t xml:space="preserve">千円</t>
     </r>
   </si>
   <si>
@@ -2221,16 +2392,73 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">1.4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">万円下がる。</t>
+      <t xml:space="preserve">1.8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円下がる。車両価格</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">100</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円ごとに</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">920</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円変動。</t>
     </r>
   </si>
   <si>
@@ -3175,7 +3403,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">（新車・年</t>
+      <t xml:space="preserve">（新車</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2,000</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円・年</t>
     </r>
     <r>
       <rPr>
@@ -3194,7 +3441,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">日）は民間実勢の上限付近（約</t>
+      <t xml:space="preserve">日）は約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円で民間実勢の上限（</t>
     </r>
     <r>
       <rPr>
@@ -3213,7 +3479,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">万円）。償却済み車両や稼働日数が多い事業者は</t>
+      <t xml:space="preserve">万円）をやや上回る。償却済み車両なら約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.6</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円で、実勢</t>
     </r>
     <r>
       <rPr>
@@ -3232,7 +3517,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">万円前後まで下げられる。</t>
+      <t xml:space="preserve">万円前後の業者はこの水準と考えられる。</t>
     </r>
   </si>
   <si>
@@ -3779,6 +4064,60 @@
   </si>
   <si>
     <t xml:space="preserve">https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">トラック流通センター 大型ダンプの価格</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.kaitoriou.net/page/knowledge/type/11679/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">GROOWAVE 10t</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダンプの価格相場</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://groowave.com/blog/truck/10t-dump/</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">SIGMA 10t</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ダンプトラック解説</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://satei.sigmaintl.jp/column/10532</t>
   </si>
   <si>
     <t xml:space="preserve">芝田建設 料金表</t>
@@ -3999,7 +4338,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -4149,6 +4488,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -4544,7 +4887,7 @@
         <v>22</v>
       </c>
       <c r="B11" s="7" t="n">
-        <v>15000000</v>
+        <v>20000000</v>
       </c>
       <c r="C11" s="6" t="s">
         <v>23</v>
@@ -5049,15 +5392,15 @@
       </c>
       <c r="C5" s="18" t="n">
         <f aca="false">(前提条件!$B$11-前提条件!$B$13)/前提条件!$B$12</f>
-        <v>2999999.8</v>
+        <v>3999999.8</v>
       </c>
       <c r="D5" s="19" t="n">
         <f aca="false">C5/前提条件!$B$6</f>
-        <v>11999.9992</v>
+        <v>15999.9992</v>
       </c>
       <c r="E5" s="20" t="n">
         <f aca="false">D5/$D$17</f>
-        <v>0.240718050392791</v>
+        <v>0.293735079797933</v>
       </c>
       <c r="F5" s="21" t="s">
         <v>90</v>
@@ -5080,7 +5423,7 @@
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">D6/$D$17</f>
-        <v>0.320957421920883</v>
+        <v>0.293735094484687</v>
       </c>
       <c r="F6" s="17" t="s">
         <v>92</v>
@@ -5103,7 +5446,7 @@
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">D7/$D$17</f>
-        <v>0.0513531875073413</v>
+        <v>0.04699761511755</v>
       </c>
       <c r="F7" s="17" t="s">
         <v>94</v>
@@ -5126,7 +5469,7 @@
       </c>
       <c r="E8" s="20" t="n">
         <f aca="false">D8/$D$17</f>
-        <v>0.00722154199321987</v>
+        <v>0.00660903962590546</v>
       </c>
       <c r="F8" s="21"/>
     </row>
@@ -5147,7 +5490,7 @@
       </c>
       <c r="E9" s="20" t="n">
         <f aca="false">D9/$D$17</f>
-        <v>0.0320957421920883</v>
+        <v>0.0293735094484687</v>
       </c>
       <c r="F9" s="21"/>
     </row>
@@ -5168,7 +5511,7 @@
       </c>
       <c r="E10" s="20" t="n">
         <f aca="false">D10/$D$17</f>
-        <v>0.0401196777401104</v>
+        <v>0.0367168868105859</v>
       </c>
       <c r="F10" s="21"/>
     </row>
@@ -5189,7 +5532,7 @@
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">D11/$D$17</f>
-        <v>0.0240718066440662</v>
+        <v>0.0220301320863516</v>
       </c>
       <c r="F11" s="21"/>
     </row>
@@ -5210,7 +5553,7 @@
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">D12/$D$17</f>
-        <v>0.00802393554802208</v>
+        <v>0.00734337736211718</v>
       </c>
       <c r="F12" s="21"/>
     </row>
@@ -5231,7 +5574,7 @@
       </c>
       <c r="E13" s="20" t="n">
         <f aca="false">D13/$D$17</f>
-        <v>0.141239501862343</v>
+        <v>0.129260131067267</v>
       </c>
       <c r="F13" s="17" t="s">
         <v>103</v>
@@ -5244,11 +5587,11 @@
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">SUM(C5:C13)</f>
-        <v>10790227.0727273</v>
+        <v>11790227.0727273</v>
       </c>
       <c r="D14" s="22" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>43160.9082909091</v>
+        <v>47160.9082909091</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">D14/$D$17</f>
@@ -5265,11 +5608,11 @@
       </c>
       <c r="C15" s="22" t="n">
         <f aca="false">C14*前提条件!$B$22</f>
-        <v>1079022.70727273</v>
+        <v>1179022.70727273</v>
       </c>
       <c r="D15" s="22" t="n">
         <f aca="false">D14*前提条件!$B$22</f>
-        <v>4316.09082909091</v>
+        <v>4716.09082909091</v>
       </c>
       <c r="E15" s="20" t="n">
         <f aca="false">D15/$D$17</f>
@@ -5288,11 +5631,11 @@
       </c>
       <c r="C16" s="22" t="n">
         <f aca="false">(C14+C15)*前提条件!$B$23</f>
-        <v>593462.489</v>
+        <v>648462.489</v>
       </c>
       <c r="D16" s="22" t="n">
         <f aca="false">(D14+D15)*前提条件!$B$23</f>
-        <v>2373.849956</v>
+        <v>2593.849956</v>
       </c>
       <c r="E16" s="20" t="n">
         <f aca="false">D16/$D$17</f>
@@ -5309,11 +5652,11 @@
       </c>
       <c r="C17" s="26" t="n">
         <f aca="false">C14+C15+C16</f>
-        <v>12462712.269</v>
+        <v>13617712.269</v>
       </c>
       <c r="D17" s="26" t="n">
         <f aca="false">D14+D15+D16</f>
-        <v>49850.849076</v>
+        <v>54470.849076</v>
       </c>
       <c r="E17" s="27" t="n">
         <f aca="false">D17/$D$17</f>
@@ -5329,7 +5672,7 @@
       <c r="C18" s="22"/>
       <c r="D18" s="22" t="n">
         <f aca="false">D17*(1+前提条件!$B$8)</f>
-        <v>54835.9339836</v>
+        <v>59917.9339836</v>
       </c>
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
@@ -5722,7 +6065,7 @@
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">A_事業者原価!$D$17</f>
-        <v>49850.849076</v>
+        <v>54470.849076</v>
       </c>
       <c r="C4" s="12" t="s">
         <v>143</v>
@@ -5813,7 +6156,7 @@
       </c>
       <c r="B12" s="18" t="n">
         <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A12+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>77663.24846</v>
+        <v>85363.24846</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A12+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
@@ -5821,7 +6164,7 @@
       </c>
       <c r="D12" s="19" t="n">
         <f aca="false">B12-C12</f>
-        <v>23099.99846</v>
+        <v>30799.99846</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5830,7 +6173,7 @@
       </c>
       <c r="B13" s="18" t="n">
         <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A13+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>60280.498845</v>
+        <v>66055.498845</v>
       </c>
       <c r="C13" s="18" t="n">
         <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A13+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
@@ -5838,7 +6181,7 @@
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">B13-C13</f>
-        <v>17324.998845</v>
+        <v>23099.998845</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5847,7 +6190,7 @@
       </c>
       <c r="B14" s="18" t="n">
         <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A14+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>54486.2489733333</v>
+        <v>59619.5823066667</v>
       </c>
       <c r="C14" s="18" t="n">
         <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A14+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
@@ -5855,7 +6198,7 @@
       </c>
       <c r="D14" s="19" t="n">
         <f aca="false">B14-C14</f>
-        <v>15399.9989733333</v>
+        <v>20533.3323066667</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5864,7 +6207,7 @@
       </c>
       <c r="B15" s="18" t="n">
         <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A15+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>49850.849076</v>
+        <v>54470.849076</v>
       </c>
       <c r="C15" s="18" t="n">
         <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A15+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
@@ -5872,7 +6215,7 @@
       </c>
       <c r="D15" s="19" t="n">
         <f aca="false">B15-C15</f>
-        <v>13859.999076</v>
+        <v>18479.999076</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5881,7 +6224,7 @@
       </c>
       <c r="B16" s="18" t="n">
         <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A16+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>46058.24916</v>
+        <v>50258.24916</v>
       </c>
       <c r="C16" s="18" t="n">
         <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A16+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
@@ -5889,7 +6232,7 @@
       </c>
       <c r="D16" s="19" t="n">
         <f aca="false">B16-C16</f>
-        <v>12599.99916</v>
+        <v>16799.99916</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5954,7 +6297,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -6051,20 +6394,44 @@
         <v>181</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="28" t="s">
+    <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="38" t="s">
+        <v>182</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="38" t="s">
+        <v>184</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="28" t="s">
+        <v>186</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="28" t="s">
         <v>151</v>
       </c>
-      <c r="B13" s="37" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="28" t="s">
-        <v>183</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>184</v>
+      <c r="B16" s="37" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="28" t="s">
+        <v>189</v>
+      </c>
+      <c r="B17" s="37" t="s">
+        <v>190</v>
       </c>
     </row>
   </sheetData>
@@ -6078,9 +6445,12 @@
     <hyperlink ref="B9" r:id="rId7" display="https://www.gov-book.or.jp/book/detail.php?product_id=408304"/>
     <hyperlink ref="B10" r:id="rId8" display="https://www.rinya.maff.go.jp/tohoku/apply/publicsale/iwatenanbu/attach/pdf/tya-ta-2-5.pdf"/>
     <hyperlink ref="B11" r:id="rId9" display="https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html"/>
-    <hyperlink ref="B12" r:id="rId10" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
-    <hyperlink ref="B13" r:id="rId11" display="https://www.matsudakougyou.com/price/"/>
-    <hyperlink ref="B14" r:id="rId12" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
+    <hyperlink ref="B12" r:id="rId10" display="https://www.kaitoriou.net/page/knowledge/type/11679/"/>
+    <hyperlink ref="B13" r:id="rId11" display="https://groowave.com/blog/truck/10t-dump/"/>
+    <hyperlink ref="B14" r:id="rId12" display="https://satei.sigmaintl.jp/column/10532"/>
+    <hyperlink ref="B15" r:id="rId13" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
+    <hyperlink ref="B16" r:id="rId14" display="https://www.matsudakougyou.com/price/"/>
+    <hyperlink ref="B17" r:id="rId15" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Base fuel cost on 270 km/day driving distance
Fuel use is now distance / fuel economy (270 km / 3.5 km/L = 77.1 L/day)
in the workbook, and the summary and detailed PDF reports are updated to
match. Also adds the standard-fare distance surcharge for 270 km.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UpX1QaVcgm2gRXfCZCnaQB
</commit_message>
<xml_diff>
--- a/research/iwate_10t_dump_cost.xlsx
+++ b/research/iwate_10t_dump_cost.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="202">
   <si>
     <r>
       <rPr>
@@ -950,6 +950,165 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">日あたり走行距離</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">km/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">指定</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ユーザー指定（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">270km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">走行）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">燃費（実走行・積載時含む）</t>
+  </si>
+  <si>
+    <t xml:space="preserve">km/L</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10t</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">車の公的積算値は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.22km/L</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">（京都府積算資料、国交省燃費一覧ベースのカタログ値）。積載・空車の往復、積込待ちのアイドリング等を考慮し実燃費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">3.5km/L</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">と仮定</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">日あたり燃料消費量</t>
     </r>
   </si>
@@ -982,64 +1141,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">標準的運賃の基礎走行</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">130km÷</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">燃費約</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.5km/L≒37L </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">と 積算基準の運転日当り約</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">58L </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">の中間</t>
+      <t xml:space="preserve">走行距離</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">÷</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">燃費</t>
     </r>
   </si>
   <si>
@@ -2363,7 +2484,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">・稼働日数・車両価格・給与が結果を大きく左右する（『比較・感度』シート参照）。償却が終わった車両なら</t>
+      <t xml:space="preserve">・稼働日数・車両価格・給与・走行距離が結果を大きく左右する（『比較・感度』シート参照）。償却が終わった車両なら</t>
     </r>
     <r>
       <rPr>
@@ -2459,6 +2580,63 @@
         <family val="2"/>
       </rPr>
       <t xml:space="preserve">円変動。</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">270km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">走行では年約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">6.8</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">となり、整備費・タイヤ費は仮定より増える可能性がある。</t>
     </r>
   </si>
   <si>
@@ -2759,7 +2937,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">）</t>
+      <t xml:space="preserve">）。公共積算は運転時間ベースのため走行距離</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">270km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">は反映しない</t>
     </r>
   </si>
   <si>
@@ -3179,7 +3376,26 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">時間制</t>
+      <t xml:space="preserve">時間制（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">130km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">以内）</t>
     </r>
   </si>
   <si>
@@ -3251,6 +3467,95 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">同上＋距離超過加算（</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日走行距離ベース）</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">130km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">超過分を</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">ごとに</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">630</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">円加算（端数切上げ）。加算額へのダンプ割増は含めない</t>
+    </r>
+  </si>
+  <si>
     <t xml:space="preserve">民間実勢（全国の料金表例）下限</t>
   </si>
   <si>
@@ -3441,17 +3746,55 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">日）は約</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">5.4</t>
+      <t xml:space="preserve">日・</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">日</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">270km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）は約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.9</t>
     </r>
     <r>
       <rPr>
@@ -3479,45 +3822,45 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">万円）をやや上回る。償却済み車両なら約</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">3.6</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">万円で、実勢</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="Arial"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">4</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color rgb="FF000000"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">万円前後の業者はこの水準と考えられる。</t>
+      <t xml:space="preserve">万円）を上回る。償却済み車両でも約</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">4.0</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">万円。民間の料金表は</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">130km</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">以内が前提のことが多く、長距離では距離加算の交渉が必要。</t>
     </r>
   </si>
   <si>
@@ -4064,6 +4407,39 @@
   </si>
   <si>
     <t xml:space="preserve">https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">京都府 積算資料（大型車の燃費</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">5.22km/L</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">）</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.pref.kyoto.jp/ryuiki/news/documents/sekisan_kizuzyo_8_12_01_b_7.pdf</t>
   </si>
   <si>
     <t xml:space="preserve">トラック流通センター 大型ダンプの価格</t>
@@ -4747,7 +5123,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -5051,262 +5427,297 @@
         <v>44</v>
       </c>
       <c r="B21" s="7" t="n">
-        <v>50</v>
+        <v>270</v>
       </c>
       <c r="C21" s="12" t="s">
         <v>45</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>11</v>
+        <v>46</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="B22" s="9" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C22" s="6"/>
+        <v>48</v>
+      </c>
+      <c r="B22" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>49</v>
+      </c>
       <c r="D22" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E22" s="6" t="s">
-        <v>48</v>
+      <c r="E22" s="12" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="B23" s="9" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="C23" s="6"/>
+      <c r="A23" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <f aca="false">B21/B22</f>
+        <v>77.1428571428571</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>52</v>
+      </c>
       <c r="D23" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B24" s="9" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E23" s="6"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="E24" s="6" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="B25" s="7" t="n">
-        <v>26900</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>52</v>
-      </c>
+        <v>56</v>
+      </c>
+      <c r="B25" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C25" s="6"/>
       <c r="D25" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>53</v>
-      </c>
+        <v>11</v>
+      </c>
+      <c r="E25" s="6"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="B26" s="13" t="n">
-        <v>5.9</v>
-      </c>
-      <c r="C26" s="12" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>56</v>
-      </c>
+      <c r="A26" s="5" t="s">
+        <v>57</v>
+      </c>
+      <c r="B26" s="2"/>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" s="11" t="n">
-        <v>246</v>
-      </c>
-      <c r="C27" s="12" t="s">
         <v>58</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <v>26900</v>
+      </c>
+      <c r="C27" s="6" t="s">
+        <v>59</v>
       </c>
       <c r="D27" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E27" s="6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="B28" s="14" t="n">
-        <v>0.04</v>
+        <v>61</v>
+      </c>
+      <c r="B28" s="13" t="n">
+        <v>5.9</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D28" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
-        <v>63</v>
-      </c>
-      <c r="B29" s="7" t="n">
-        <v>22147</v>
-      </c>
-      <c r="C29" s="6" t="s">
         <v>64</v>
+      </c>
+      <c r="B29" s="11" t="n">
+        <v>246</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>65</v>
       </c>
       <c r="D29" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="B30" s="11" t="n">
-        <v>180</v>
-      </c>
-      <c r="C30" s="6" t="s">
         <v>67</v>
+      </c>
+      <c r="B30" s="14" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>68</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="B31" s="11" t="n">
-        <v>140</v>
+        <v>70</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <v>22147</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D31" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="B32" s="15" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C32" s="6"/>
+        <v>73</v>
+      </c>
+      <c r="B32" s="11" t="n">
+        <v>180</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>74</v>
+      </c>
       <c r="D32" s="6" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="B33" s="2"/>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="A33" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B33" s="11" t="n">
+        <v>140</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D33" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="6" t="s">
-        <v>73</v>
-      </c>
-      <c r="B34" s="11" t="n">
-        <v>52610</v>
-      </c>
-      <c r="C34" s="6" t="s">
-        <v>23</v>
-      </c>
+        <v>77</v>
+      </c>
+      <c r="B34" s="15" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C34" s="6"/>
       <c r="D34" s="6" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="B35" s="9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C35" s="6"/>
-      <c r="D35" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>76</v>
-      </c>
+      <c r="A35" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" s="2"/>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="6" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B36" s="11" t="n">
-        <v>3130</v>
+        <v>52610</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>78</v>
+        <v>23</v>
       </c>
       <c r="D36" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>68</v>
+        <v>81</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B37" s="11" t="n">
-        <v>630</v>
-      </c>
-      <c r="C37" s="6" t="s">
-        <v>80</v>
-      </c>
+        <v>82</v>
+      </c>
+      <c r="B37" s="9" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C37" s="6"/>
       <c r="D37" s="6" t="s">
         <v>15</v>
       </c>
       <c r="E37" s="6" t="s">
-        <v>68</v>
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B38" s="11" t="n">
+        <v>3130</v>
+      </c>
+      <c r="C38" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="B39" s="11" t="n">
+        <v>630</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="E39" s="6" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -5337,7 +5748,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5347,7 +5758,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5368,27 +5779,27 @@
         <v>6</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D4" s="16" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C5" s="18" t="n">
         <f aca="false">(前提条件!$B$11-前提条件!$B$13)/前提条件!$B$12</f>
@@ -5400,18 +5811,18 @@
       </c>
       <c r="E5" s="20" t="n">
         <f aca="false">D5/$D$17</f>
-        <v>0.293735079797933</v>
+        <v>0.271713740242734</v>
       </c>
       <c r="F5" s="21" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="C6" s="18" t="n">
         <f aca="false">前提条件!$B$14</f>
@@ -5423,18 +5834,18 @@
       </c>
       <c r="E6" s="20" t="n">
         <f aca="false">D6/$D$17</f>
-        <v>0.293735094484687</v>
+        <v>0.271713753828421</v>
       </c>
       <c r="F6" s="17" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C7" s="18" t="n">
         <f aca="false">前提条件!$B$14*前提条件!$B$15</f>
@@ -5446,18 +5857,18 @@
       </c>
       <c r="E7" s="20" t="n">
         <f aca="false">D7/$D$17</f>
-        <v>0.04699761511755</v>
+        <v>0.0434742006125474</v>
       </c>
       <c r="F7" s="17" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="C8" s="18" t="n">
         <f aca="false">前提条件!$B$16</f>
@@ -5469,16 +5880,16 @@
       </c>
       <c r="E8" s="20" t="n">
         <f aca="false">D8/$D$17</f>
-        <v>0.00660903962590546</v>
+        <v>0.00611355946113948</v>
       </c>
       <c r="F8" s="21"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C9" s="18" t="n">
         <f aca="false">前提条件!$B$17</f>
@@ -5490,16 +5901,16 @@
       </c>
       <c r="E9" s="20" t="n">
         <f aca="false">D9/$D$17</f>
-        <v>0.0293735094484687</v>
+        <v>0.0271713753828421</v>
       </c>
       <c r="F9" s="21"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C10" s="18" t="n">
         <f aca="false">前提条件!$B$18</f>
@@ -5511,16 +5922,16 @@
       </c>
       <c r="E10" s="20" t="n">
         <f aca="false">D10/$D$17</f>
-        <v>0.0367168868105859</v>
+        <v>0.0339642192285527</v>
       </c>
       <c r="F10" s="21"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C11" s="18" t="n">
         <f aca="false">前提条件!$B$19</f>
@@ -5532,16 +5943,16 @@
       </c>
       <c r="E11" s="20" t="n">
         <f aca="false">D11/$D$17</f>
-        <v>0.0220301320863516</v>
+        <v>0.0203785315371316</v>
       </c>
       <c r="F11" s="21"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="C12" s="18" t="n">
         <f aca="false">前提条件!$B$20</f>
@@ -5553,45 +5964,45 @@
       </c>
       <c r="E12" s="20" t="n">
         <f aca="false">D12/$D$17</f>
-        <v>0.00734337736211718</v>
+        <v>0.00679284384571054</v>
       </c>
       <c r="F12" s="21"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C13" s="18" t="n">
-        <f aca="false">前提条件!$B$21*前提条件!$B$9*前提条件!$B$6</f>
-        <v>1760227.27272727</v>
+        <f aca="false">前提条件!$B$23*前提条件!$B$9*前提条件!$B$6</f>
+        <v>2715779.22077922</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">C13/前提条件!$B$6</f>
-        <v>7040.90909090909</v>
+        <v>10863.1168831169</v>
       </c>
       <c r="E13" s="20" t="n">
         <f aca="false">D13/$D$17</f>
-        <v>0.129260131067267</v>
+        <v>0.184478641661787</v>
       </c>
       <c r="F13" s="17" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21"/>
       <c r="B14" s="17" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="C14" s="22" t="n">
         <f aca="false">SUM(C5:C13)</f>
-        <v>11790227.0727273</v>
+        <v>12745779.0207792</v>
       </c>
       <c r="D14" s="22" t="n">
         <f aca="false">SUM(D5:D13)</f>
-        <v>47160.9082909091</v>
+        <v>50983.1160831169</v>
       </c>
       <c r="E14" s="23" t="n">
         <f aca="false">D14/$D$17</f>
@@ -5601,62 +6012,62 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C15" s="22" t="n">
-        <f aca="false">C14*前提条件!$B$22</f>
-        <v>1179022.70727273</v>
+        <f aca="false">C14*前提条件!$B$24</f>
+        <v>1274577.90207792</v>
       </c>
       <c r="D15" s="22" t="n">
-        <f aca="false">D14*前提条件!$B$22</f>
-        <v>4716.09082909091</v>
+        <f aca="false">D14*前提条件!$B$24</f>
+        <v>5098.31160831169</v>
       </c>
       <c r="E15" s="20" t="n">
         <f aca="false">D15/$D$17</f>
         <v>0.0865800865800866</v>
       </c>
       <c r="F15" s="17" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C16" s="22" t="n">
-        <f aca="false">(C14+C15)*前提条件!$B$23</f>
-        <v>648462.489</v>
+        <f aca="false">(C14+C15)*前提条件!$B$25</f>
+        <v>701017.846142857</v>
       </c>
       <c r="D16" s="22" t="n">
-        <f aca="false">(D14+D15)*前提条件!$B$23</f>
-        <v>2593.849956</v>
+        <f aca="false">(D14+D15)*前提条件!$B$25</f>
+        <v>2804.07138457143</v>
       </c>
       <c r="E16" s="20" t="n">
         <f aca="false">D16/$D$17</f>
         <v>0.0476190476190476</v>
       </c>
       <c r="F16" s="21" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="24"/>
       <c r="B17" s="25" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C17" s="26" t="n">
         <f aca="false">C14+C15+C16</f>
-        <v>13617712.269</v>
+        <v>14721374.769</v>
       </c>
       <c r="D17" s="26" t="n">
         <f aca="false">D14+D15+D16</f>
-        <v>54470.849076</v>
+        <v>58885.499076</v>
       </c>
       <c r="E17" s="27" t="n">
         <f aca="false">D17/$D$17</f>
@@ -5667,12 +6078,12 @@
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21"/>
       <c r="B18" s="17" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="C18" s="22"/>
       <c r="D18" s="22" t="n">
         <f aca="false">D17*(1+前提条件!$B$8)</f>
-        <v>59917.9339836</v>
+        <v>64774.0489836</v>
       </c>
       <c r="E18" s="21"/>
       <c r="F18" s="21"/>
@@ -5687,7 +6098,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -5697,7 +6108,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -5707,7 +6118,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
@@ -5717,7 +6128,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="28" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B23" s="2"/>
       <c r="C23" s="2"/>
@@ -5755,7 +6166,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5766,7 +6177,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -5786,40 +6197,40 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B5" s="29" t="n">
         <f aca="false">1</f>
         <v>1</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D5" s="30" t="n">
-        <f aca="false">前提条件!$B$25</f>
+        <f aca="false">前提条件!$B$27</f>
         <v>26900</v>
       </c>
       <c r="E5" s="19" t="n">
@@ -5831,19 +6242,19 @@
         <v>0.352740320844015</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B6" s="31" t="n">
-        <f aca="false">前提条件!$B$27*前提条件!$B$28*前提条件!$B$26</f>
+        <f aca="false">前提条件!$B$29*前提条件!$B$30*前提条件!$B$28</f>
         <v>58.056</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D6" s="30" t="n">
         <f aca="false">前提条件!$B$9</f>
@@ -5858,22 +6269,22 @@
         <v>0.107203426872793</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B7" s="31" t="n">
-        <f aca="false">前提条件!$B$30/前提条件!$B$31</f>
+        <f aca="false">前提条件!$B$32/前提条件!$B$33</f>
         <v>1.28571428571429</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="D7" s="30" t="n">
-        <f aca="false">前提条件!$B$29</f>
+        <f aca="false">前提条件!$B$31</f>
         <v>22147</v>
       </c>
       <c r="E7" s="19" t="n">
@@ -5885,12 +6296,12 @@
         <v>0.373389585616525</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="32" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B8" s="21"/>
       <c r="C8" s="21"/>
@@ -5907,13 +6318,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B9" s="21"/>
       <c r="C9" s="21"/>
       <c r="D9" s="21"/>
       <c r="E9" s="19" t="n">
-        <f aca="false">E8*前提条件!$B$32</f>
+        <f aca="false">E8*前提条件!$B$34</f>
         <v>12710.0109298701</v>
       </c>
       <c r="F9" s="20" t="n">
@@ -5921,12 +6332,12 @@
         <v>0.166666666666667</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="34" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B10" s="24"/>
       <c r="C10" s="24"/>
@@ -5943,7 +6354,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B11" s="21"/>
       <c r="C11" s="21"/>
@@ -5966,7 +6377,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" s="2"/>
@@ -5977,7 +6388,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="28" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" s="2"/>
@@ -5988,7 +6399,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="28" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" s="2"/>
@@ -5999,7 +6410,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" s="2"/>
@@ -6024,7 +6435,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
@@ -6035,7 +6446,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -6049,209 +6460,214 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C3" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D3" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="B4" s="18" t="n">
         <f aca="false">A_事業者原価!$D$17</f>
-        <v>54470.849076</v>
+        <v>58885.499076</v>
       </c>
       <c r="C4" s="12" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="D4" s="2"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="B5" s="18" t="n">
         <f aca="false">B_公共積算!$E$10</f>
         <v>76260.0655792208</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B6" s="18" t="n">
-        <f aca="false">前提条件!$B$34*(1+前提条件!$B$35)</f>
+        <f aca="false">前提条件!$B$36*(1+前提条件!$B$37)</f>
         <v>63132</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>148</v>
-      </c>
-      <c r="B7" s="11" t="n">
-        <v>36000</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>149</v>
+        <v>155</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <f aca="false">前提条件!$B$36*(1+前提条件!$B$37)+ROUNDUP(MAX(0,前提条件!$B$21-130)/10,0)*前提条件!$B$39</f>
+        <v>71952</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>156</v>
       </c>
       <c r="D7" s="2"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="B8" s="11" t="n">
+        <v>36000</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>158</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
+        <v>159</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <v>50000</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
+      <c r="C9" s="6" t="s">
+        <v>160</v>
+      </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
-        <v>152</v>
-      </c>
+      <c r="A10" s="2"/>
       <c r="B10" s="2"/>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="4" t="s">
+      <c r="A11" s="5" t="s">
+        <v>161</v>
+      </c>
+      <c r="B11" s="2"/>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C11" s="4" t="s">
-        <v>154</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="36" t="n">
-        <v>150</v>
-      </c>
-      <c r="B12" s="18" t="n">
-        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A12+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>85363.24846</v>
-      </c>
-      <c r="C12" s="18" t="n">
-        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A12+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>54563.25</v>
-      </c>
-      <c r="D12" s="19" t="n">
-        <f aca="false">B12-C12</f>
-        <v>30799.99846</v>
+      <c r="B12" s="4" t="s">
+        <v>162</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>163</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="36" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="B13" s="18" t="n">
-        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A13+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>66055.498845</v>
+        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A13+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>89777.89846</v>
       </c>
       <c r="C13" s="18" t="n">
-        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A13+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>42955.5</v>
+        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A13+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>58977.9</v>
       </c>
       <c r="D13" s="19" t="n">
         <f aca="false">B13-C13</f>
-        <v>23099.998845</v>
+        <v>30799.99846</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="36" t="n">
-        <v>225</v>
+        <v>200</v>
       </c>
       <c r="B14" s="18" t="n">
-        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A14+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>59619.5823066667</v>
+        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A14+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>70470.148845</v>
       </c>
       <c r="C14" s="18" t="n">
-        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A14+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>39086.25</v>
+        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A14+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>47370.15</v>
       </c>
       <c r="D14" s="19" t="n">
         <f aca="false">B14-C14</f>
-        <v>20533.3323066667</v>
+        <v>23099.998845</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="36" t="n">
-        <v>250</v>
+        <v>225</v>
       </c>
       <c r="B15" s="18" t="n">
-        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A15+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>54470.849076</v>
+        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A15+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>64034.2323066667</v>
       </c>
       <c r="C15" s="18" t="n">
-        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A15+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>35990.85</v>
+        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A15+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>43500.9</v>
       </c>
       <c r="D15" s="19" t="n">
         <f aca="false">B15-C15</f>
-        <v>18479.999076</v>
+        <v>20533.3323066667</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="36" t="n">
-        <v>275</v>
+        <v>250</v>
       </c>
       <c r="B16" s="18" t="n">
-        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A16+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>50258.24916</v>
+        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A16+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>58885.499076</v>
       </c>
       <c r="C16" s="18" t="n">
-        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A16+(前提条件!$B$21*前提条件!$B$9))*(1+前提条件!$B$22)*(1+前提条件!$B$23)</f>
-        <v>33458.25</v>
+        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A16+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>40405.5</v>
       </c>
       <c r="D16" s="19" t="n">
         <f aca="false">B16-C16</f>
+        <v>18479.999076</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="36" t="n">
+        <v>275</v>
+      </c>
+      <c r="B17" s="18" t="n">
+        <f aca="false">(SUM(A_事業者原価!$C$5:$C$12)/A17+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>54672.89916</v>
+      </c>
+      <c r="C17" s="18" t="n">
+        <f aca="false">((SUM(A_事業者原価!$C$5:$C$12)-A_事業者原価!$C$5)/A17+(前提条件!$B$23*前提条件!$B$9))*(1+前提条件!$B$24)*(1+前提条件!$B$25)</f>
+        <v>37872.9</v>
+      </c>
+      <c r="D17" s="19" t="n">
+        <f aca="false">B17-C17</f>
         <v>16799.99916</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
-    </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>156</v>
-      </c>
+      <c r="A18" s="2"/>
       <c r="B18" s="2"/>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
-        <v>157</v>
+      <c r="A19" s="5" t="s">
+        <v>165</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" s="2"/>
@@ -6259,7 +6675,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="28" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
@@ -6267,7 +6683,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="28" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="B21" s="2"/>
       <c r="C21" s="2"/>
@@ -6275,11 +6691,19 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="28" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="B23" s="2"/>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -6297,7 +6721,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -6306,7 +6730,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B1" s="2"/>
     </row>
@@ -6316,122 +6740,130 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="B3" s="37" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="28" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="B4" s="37" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="28" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>167</v>
+        <v>176</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="28" t="s">
-        <v>168</v>
+        <v>177</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="28" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="B7" s="37" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="28" t="s">
-        <v>172</v>
+        <v>181</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>173</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="28" t="s">
-        <v>174</v>
+        <v>183</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>175</v>
+        <v>184</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="28" t="s">
-        <v>176</v>
+        <v>185</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="28" t="s">
-        <v>178</v>
+        <v>187</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="28" t="s">
-        <v>180</v>
+        <v>189</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="38" t="s">
-        <v>182</v>
+        <v>190</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="28" t="s">
+        <v>191</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>183</v>
+        <v>192</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="38" t="s">
-        <v>184</v>
+        <v>193</v>
       </c>
       <c r="B14" s="37" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="28" t="s">
-        <v>186</v>
+        <v>194</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="14.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="38" t="s">
+        <v>195</v>
       </c>
       <c r="B15" s="37" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="28" t="s">
-        <v>151</v>
+        <v>197</v>
       </c>
       <c r="B16" s="37" t="s">
-        <v>188</v>
+        <v>198</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="28" t="s">
-        <v>189</v>
+        <v>160</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>190</v>
+        <v>199</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -6445,12 +6877,13 @@
     <hyperlink ref="B9" r:id="rId7" display="https://www.gov-book.or.jp/book/detail.php?product_id=408304"/>
     <hyperlink ref="B10" r:id="rId8" display="https://www.rinya.maff.go.jp/tohoku/apply/publicsale/iwatenanbu/attach/pdf/tya-ta-2-5.pdf"/>
     <hyperlink ref="B11" r:id="rId9" display="https://oil-stat.com/light/%E5%B2%A9%E6%89%8B%E7%9C%8C.html"/>
-    <hyperlink ref="B12" r:id="rId10" display="https://www.kaitoriou.net/page/knowledge/type/11679/"/>
-    <hyperlink ref="B13" r:id="rId11" display="https://groowave.com/blog/truck/10t-dump/"/>
-    <hyperlink ref="B14" r:id="rId12" display="https://satei.sigmaintl.jp/column/10532"/>
-    <hyperlink ref="B15" r:id="rId13" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
-    <hyperlink ref="B16" r:id="rId14" display="https://www.matsudakougyou.com/price/"/>
-    <hyperlink ref="B17" r:id="rId15" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
+    <hyperlink ref="B12" r:id="rId10" display="https://www.pref.kyoto.jp/ryuiki/news/documents/sekisan_kizuzyo_8_12_01_b_7.pdf"/>
+    <hyperlink ref="B13" r:id="rId11" display="https://www.kaitoriou.net/page/knowledge/type/11679/"/>
+    <hyperlink ref="B14" r:id="rId12" display="https://groowave.com/blog/truck/10t-dump/"/>
+    <hyperlink ref="B15" r:id="rId13" display="https://satei.sigmaintl.jp/column/10532"/>
+    <hyperlink ref="B16" r:id="rId14" display="http://shibata3000.com/wp/wp-content/uploads/rental_pricelist.pdf"/>
+    <hyperlink ref="B17" r:id="rId15" display="https://www.matsudakougyou.com/price/"/>
+    <hyperlink ref="B18" r:id="rId16" display="https://xn--pckua2a7gp15o89zb.com/%E3%83%80%E3%83%B3%E3%83%97%E9%81%8B%E8%BB%A2%E6%89%8B%E3%81%AE%E4%BB%95%E4%BA%8B-%E5%B2%A9%E6%89%8B%E7%9C%8C"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>